<commit_message>
fix robustness of task verification
</commit_message>
<xml_diff>
--- a/tasks/finalpool/arxiv-research-pipeline-notion-excel/groundtruth_workspace/Research_Knowledge_Base.xlsx
+++ b/tasks/finalpool/arxiv-research-pipeline-notion-excel/groundtruth_workspace/Research_Knowledge_Base.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -532,6 +532,62 @@
       </c>
       <c r="F4" t="n">
         <v>120</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2304.00004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Chain-of-Thought Reasoning in Large Language Models</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Author F</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cs.CL</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2305.00005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Survey of In-Context Learning for Large Language Models</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Author G</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>cs.LG</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>